<commit_message>
feat: implement source tier multipliers, boost TGC/DG/Ligonier/9Marks to 1.3x, Jen Wilkin/Kyle Worley/American Reformer promoted
</commit_message>
<xml_diff>
--- a/scoring_algorithm.xlsx
+++ b/scoring_algorithm.xlsx
@@ -230,7 +230,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -380,6 +380,63 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1597,8 +1654,8 @@
     <mergeCell ref="A62:D62"/>
     <mergeCell ref="C14:D14"/>
     <mergeCell ref="C45:D45"/>
+    <mergeCell ref="A28:D28"/>
     <mergeCell ref="C26:D26"/>
-    <mergeCell ref="A28:D28"/>
     <mergeCell ref="C64:D64"/>
     <mergeCell ref="A13:D13"/>
     <mergeCell ref="B10:D10"/>
@@ -1701,678 +1758,678 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="26" t="inlineStr">
+    <row r="5" ht="36" customHeight="1">
+      <c r="A5" s="52" t="inlineStr">
         <is>
           <t>The Gospel Coalition</t>
         </is>
       </c>
-      <c r="B5" s="27" t="inlineStr">
+      <c r="B5" s="53" t="inlineStr">
+        <is>
+          <t>Tier 1A</t>
+        </is>
+      </c>
+      <c r="C5" s="53" t="inlineStr">
+        <is>
+          <t>1.30×</t>
+        </is>
+      </c>
+      <c r="D5" s="54" t="inlineStr">
+        <is>
+          <t>Christian</t>
+        </is>
+      </c>
+      <c r="E5" s="55" t="inlineStr">
+        <is>
+          <t>Premier Reformed evangelical outlet. Elevated to 1.3x for editorial excellence and wide readership.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="52" t="inlineStr">
+        <is>
+          <t>Desiring God</t>
+        </is>
+      </c>
+      <c r="B6" s="53" t="inlineStr">
+        <is>
+          <t>Tier 1A</t>
+        </is>
+      </c>
+      <c r="C6" s="53" t="inlineStr">
+        <is>
+          <t>1.30×</t>
+        </is>
+      </c>
+      <c r="D6" s="54" t="inlineStr">
+        <is>
+          <t>Christian</t>
+        </is>
+      </c>
+      <c r="E6" s="55" t="inlineStr">
+        <is>
+          <t>John Piper's ministry. Deeply theological and devotional. Elevated to 1.3x.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="52" t="inlineStr">
+        <is>
+          <t>Ligonier Ministries</t>
+        </is>
+      </c>
+      <c r="B7" s="53" t="inlineStr">
+        <is>
+          <t>Tier 1A</t>
+        </is>
+      </c>
+      <c r="C7" s="53" t="inlineStr">
+        <is>
+          <t>1.30×</t>
+        </is>
+      </c>
+      <c r="D7" s="54" t="inlineStr">
+        <is>
+          <t>Christian</t>
+        </is>
+      </c>
+      <c r="E7" s="55" t="inlineStr">
+        <is>
+          <t>R.C. Sproul's legacy. Reformed theology, serious biblical exposition. Elevated to 1.3x.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="52" t="inlineStr">
+        <is>
+          <t>9Marks</t>
+        </is>
+      </c>
+      <c r="B8" s="53" t="inlineStr">
+        <is>
+          <t>Tier 1A</t>
+        </is>
+      </c>
+      <c r="C8" s="53" t="inlineStr">
+        <is>
+          <t>1.30×</t>
+        </is>
+      </c>
+      <c r="D8" s="54" t="inlineStr">
+        <is>
+          <t>Christian</t>
+        </is>
+      </c>
+      <c r="E8" s="55" t="inlineStr">
+        <is>
+          <t>Church health and polity. Deeply practical for pastors. Elevated to 1.3x.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="36" customHeight="1">
+      <c r="A9" s="56" t="inlineStr">
+        <is>
+          <t>Christianity Today</t>
+        </is>
+      </c>
+      <c r="B9" s="57" t="inlineStr">
         <is>
           <t>Tier 1</t>
         </is>
       </c>
-      <c r="C5" s="27" t="inlineStr">
+      <c r="C9" s="57" t="inlineStr">
         <is>
           <t>1.20×</t>
         </is>
       </c>
-      <c r="D5" s="28" t="inlineStr">
+      <c r="D9" s="58" t="inlineStr">
         <is>
           <t>Christian</t>
         </is>
       </c>
-      <c r="E5" s="29" t="inlineStr">
-        <is>
-          <t>Premier Reformed evangelical outlet. Strong editorial standards, theologically robust, wide readership. Flagship source.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="30" t="inlineStr">
-        <is>
-          <t>Christianity Today</t>
-        </is>
-      </c>
-      <c r="B6" s="27" t="inlineStr">
+      <c r="E9" s="59" t="inlineStr">
+        <is>
+          <t>Flagship evangelical magazine. Broad evangelical coverage, strong long-form.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="56" t="inlineStr">
+        <is>
+          <t>First Things</t>
+        </is>
+      </c>
+      <c r="B10" s="57" t="inlineStr">
         <is>
           <t>Tier 1</t>
         </is>
       </c>
-      <c r="C6" s="27" t="inlineStr">
+      <c r="C10" s="57" t="inlineStr">
         <is>
           <t>1.20×</t>
         </is>
       </c>
-      <c r="D6" s="31" t="inlineStr">
+      <c r="D10" s="58" t="inlineStr">
         <is>
           <t>Christian</t>
         </is>
       </c>
-      <c r="E6" s="32" t="inlineStr">
-        <is>
-          <t>Flagship evangelical magazine since 1956. Broad evangelical coverage, strong reporting and long-form essays.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="26" t="inlineStr">
-        <is>
-          <t>Desiring God</t>
-        </is>
-      </c>
-      <c r="B7" s="27" t="inlineStr">
+      <c r="E10" s="59" t="inlineStr">
+        <is>
+          <t>Premier journal of religion and public life. High literary and theological quality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="56" t="inlineStr">
+        <is>
+          <t>Crossway</t>
+        </is>
+      </c>
+      <c r="B11" s="57" t="inlineStr">
         <is>
           <t>Tier 1</t>
         </is>
       </c>
-      <c r="C7" s="27" t="inlineStr">
+      <c r="C11" s="57" t="inlineStr">
         <is>
           <t>1.20×</t>
         </is>
       </c>
-      <c r="D7" s="28" t="inlineStr">
+      <c r="D11" s="58" t="inlineStr">
         <is>
           <t>Christian</t>
         </is>
       </c>
-      <c r="E7" s="29" t="inlineStr">
-        <is>
-          <t>John Piper's ministry. Deeply theological, devotional, and pastoral content. Very high quality for Reformed readers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="30" t="inlineStr">
-        <is>
-          <t>Ligonier Ministries</t>
-        </is>
-      </c>
-      <c r="B8" s="27" t="inlineStr">
+      <c r="E11" s="59" t="inlineStr">
+        <is>
+          <t>Publisher blog. Theological depth, features leading evangelical authors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="36" customHeight="1">
+      <c r="A12" s="56" t="inlineStr">
+        <is>
+          <t>Mere Orthodoxy</t>
+        </is>
+      </c>
+      <c r="B12" s="57" t="inlineStr">
         <is>
           <t>Tier 1</t>
         </is>
       </c>
-      <c r="C8" s="27" t="inlineStr">
+      <c r="C12" s="57" t="inlineStr">
         <is>
           <t>1.20×</t>
         </is>
       </c>
-      <c r="D8" s="31" t="inlineStr">
+      <c r="D12" s="58" t="inlineStr">
         <is>
           <t>Christian</t>
         </is>
       </c>
-      <c r="E8" s="32" t="inlineStr">
-        <is>
-          <t>R.C. Sproul's legacy ministry. Reformed theology, serious biblical exposition. Excellent for theologically minded readers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="40" customHeight="1">
-      <c r="A9" s="26" t="inlineStr">
-        <is>
-          <t>First Things</t>
-        </is>
-      </c>
-      <c r="B9" s="27" t="inlineStr">
+      <c r="E12" s="59" t="inlineStr">
+        <is>
+          <t>Thoughtful, intellectually serious. Best independent evangelical outlet online.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="36" customHeight="1">
+      <c r="A13" s="56" t="inlineStr">
+        <is>
+          <t>American Reformer</t>
+        </is>
+      </c>
+      <c r="B13" s="57" t="inlineStr">
         <is>
           <t>Tier 1</t>
         </is>
       </c>
-      <c r="C9" s="27" t="inlineStr">
+      <c r="C13" s="57" t="inlineStr">
         <is>
           <t>1.20×</t>
         </is>
       </c>
-      <c r="D9" s="28" t="inlineStr">
+      <c r="D13" s="58" t="inlineStr">
         <is>
           <t>Christian</t>
         </is>
       </c>
-      <c r="E9" s="29" t="inlineStr">
-        <is>
-          <t>Premier journal of religion and public life. Serious, intellectual, ecumenical. High literary and theological quality.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="40" customHeight="1">
-      <c r="A10" s="30" t="inlineStr">
-        <is>
-          <t>9Marks</t>
-        </is>
-      </c>
-      <c r="B10" s="27" t="inlineStr">
-        <is>
-          <t>Tier 1</t>
-        </is>
-      </c>
-      <c r="C10" s="27" t="inlineStr">
-        <is>
-          <t>1.20×</t>
-        </is>
-      </c>
-      <c r="D10" s="31" t="inlineStr">
+      <c r="E13" s="59" t="inlineStr">
+        <is>
+          <t>Elevated to Tier 1. Strong Reformed cultural commentary with consistent editorial quality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="36" customHeight="1">
+      <c r="A14" s="60" t="inlineStr">
+        <is>
+          <t>World Magazine</t>
+        </is>
+      </c>
+      <c r="B14" s="61" t="inlineStr">
+        <is>
+          <t>Tier 2</t>
+        </is>
+      </c>
+      <c r="C14" s="61" t="inlineStr">
+        <is>
+          <t>1.05×</t>
+        </is>
+      </c>
+      <c r="D14" s="62" t="inlineStr">
         <is>
           <t>Christian</t>
         </is>
       </c>
-      <c r="E10" s="32" t="inlineStr">
-        <is>
-          <t>Focused on church health and polity. Deeply practical for pastors and church leaders. Niche but excellent.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="26" t="inlineStr">
-        <is>
-          <t>Crossway</t>
-        </is>
-      </c>
-      <c r="B11" s="27" t="inlineStr">
-        <is>
-          <t>Tier 1</t>
-        </is>
-      </c>
-      <c r="C11" s="27" t="inlineStr">
-        <is>
-          <t>1.20×</t>
-        </is>
-      </c>
-      <c r="D11" s="28" t="inlineStr">
+      <c r="E14" s="63" t="inlineStr">
+        <is>
+          <t>Strong Reformed news reporting. Trustworthy, consistent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="36" customHeight="1">
+      <c r="A15" s="60" t="inlineStr">
+        <is>
+          <t>Relevant Magazine</t>
+        </is>
+      </c>
+      <c r="B15" s="61" t="inlineStr">
+        <is>
+          <t>Tier 2</t>
+        </is>
+      </c>
+      <c r="C15" s="61" t="inlineStr">
+        <is>
+          <t>1.05×</t>
+        </is>
+      </c>
+      <c r="D15" s="62" t="inlineStr">
         <is>
           <t>Christian</t>
         </is>
       </c>
-      <c r="E11" s="29" t="inlineStr">
-        <is>
-          <t>Publisher with strong editorial blog. Theological depth, often features leading evangelical authors.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="40" customHeight="1">
-      <c r="A12" s="30" t="inlineStr">
-        <is>
-          <t>Mere Orthodoxy</t>
-        </is>
-      </c>
-      <c r="B12" s="27" t="inlineStr">
-        <is>
-          <t>Tier 1</t>
-        </is>
-      </c>
-      <c r="C12" s="27" t="inlineStr">
-        <is>
-          <t>1.20×</t>
-        </is>
-      </c>
-      <c r="D12" s="31" t="inlineStr">
+      <c r="E15" s="63" t="inlineStr">
+        <is>
+          <t>Younger evangelical audience. Culture-focused. Good for seeker and student personas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="36" customHeight="1">
+      <c r="A16" s="60" t="inlineStr">
+        <is>
+          <t>Reformation21</t>
+        </is>
+      </c>
+      <c r="B16" s="61" t="inlineStr">
+        <is>
+          <t>Tier 2</t>
+        </is>
+      </c>
+      <c r="C16" s="61" t="inlineStr">
+        <is>
+          <t>1.05×</t>
+        </is>
+      </c>
+      <c r="D16" s="62" t="inlineStr">
         <is>
           <t>Christian</t>
         </is>
       </c>
-      <c r="E12" s="32" t="inlineStr">
-        <is>
-          <t>Thoughtful, intellectually serious. Best independent evangelical outlet online. Punches above its weight.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="26" t="inlineStr">
-        <is>
-          <t>World Magazine</t>
-        </is>
-      </c>
-      <c r="B13" s="33" t="inlineStr">
+      <c r="E16" s="63" t="inlineStr">
+        <is>
+          <t>Alliance of Confessing Evangelicals. Solid Reformed theology.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="36" customHeight="1">
+      <c r="A17" s="60" t="inlineStr">
+        <is>
+          <t>Jen Wilkin</t>
+        </is>
+      </c>
+      <c r="B17" s="61" t="inlineStr">
         <is>
           <t>Tier 2</t>
         </is>
       </c>
-      <c r="C13" s="33" t="inlineStr">
+      <c r="C17" s="61" t="inlineStr">
         <is>
           <t>1.05×</t>
         </is>
       </c>
-      <c r="D13" s="28" t="inlineStr">
-        <is>
-          <t>Christian</t>
-        </is>
-      </c>
-      <c r="E13" s="29" t="inlineStr">
-        <is>
-          <t>Strong Reformed news reporting. Trustworthy, consistent, but more news-oriented than essay-driven.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="40" customHeight="1">
-      <c r="A14" s="30" t="inlineStr">
-        <is>
-          <t>Relevant Magazine</t>
-        </is>
-      </c>
-      <c r="B14" s="33" t="inlineStr">
+      <c r="D17" s="62" t="inlineStr">
+        <is>
+          <t>Author Substack</t>
+        </is>
+      </c>
+      <c r="E17" s="63" t="inlineStr">
+        <is>
+          <t>Elevated to Tier 2. Bible teacher and author with consistently high-quality content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="36" customHeight="1">
+      <c r="A18" s="60" t="inlineStr">
+        <is>
+          <t>Kyle Worley</t>
+        </is>
+      </c>
+      <c r="B18" s="61" t="inlineStr">
         <is>
           <t>Tier 2</t>
         </is>
       </c>
-      <c r="C14" s="33" t="inlineStr">
+      <c r="C18" s="61" t="inlineStr">
         <is>
           <t>1.05×</t>
         </is>
       </c>
-      <c r="D14" s="31" t="inlineStr">
-        <is>
-          <t>Christian</t>
-        </is>
-      </c>
-      <c r="E14" s="32" t="inlineStr">
-        <is>
-          <t>Younger evangelical audience. Culture-focused. Good for seeker and student personas. Lighter theological depth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="26" t="inlineStr">
-        <is>
-          <t>American Reformer</t>
-        </is>
-      </c>
-      <c r="B15" s="33" t="inlineStr">
-        <is>
-          <t>Tier 2</t>
-        </is>
-      </c>
-      <c r="C15" s="33" t="inlineStr">
-        <is>
-          <t>1.05×</t>
-        </is>
-      </c>
-      <c r="D15" s="28" t="inlineStr">
-        <is>
-          <t>Christian</t>
-        </is>
-      </c>
-      <c r="E15" s="29" t="inlineStr">
-        <is>
-          <t>Conservative Reformed cultural commentary. Strong perspective but narrower audience. Worth watching.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="40" customHeight="1">
-      <c r="A16" s="30" t="inlineStr">
-        <is>
-          <t>Reformation21</t>
-        </is>
-      </c>
-      <c r="B16" s="33" t="inlineStr">
-        <is>
-          <t>Tier 2</t>
-        </is>
-      </c>
-      <c r="C16" s="33" t="inlineStr">
-        <is>
-          <t>1.05×</t>
-        </is>
-      </c>
-      <c r="D16" s="31" t="inlineStr">
-        <is>
-          <t>Christian</t>
-        </is>
-      </c>
-      <c r="E16" s="32" t="inlineStr">
-        <is>
-          <t>Alliance of Confessing Evangelicals. Solid Reformed theology. Smaller readership but high quality.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="40" customHeight="1">
-      <c r="A17" s="26" t="inlineStr">
+      <c r="D18" s="62" t="inlineStr">
+        <is>
+          <t>Author Substack</t>
+        </is>
+      </c>
+      <c r="E18" s="63" t="inlineStr">
+        <is>
+          <t>Elevated to Tier 2. Pastor/theologian with theologically solid, pastoral writing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="36" customHeight="1">
+      <c r="A19" s="64" t="inlineStr">
         <is>
           <t>Karen Swallow Prior</t>
         </is>
       </c>
-      <c r="B17" s="18" t="inlineStr">
+      <c r="B19" s="65" t="inlineStr">
         <is>
           <t>Tier 3</t>
         </is>
       </c>
-      <c r="C17" s="18" t="inlineStr">
+      <c r="C19" s="65" t="inlineStr">
         <is>
           <t>1.00×</t>
         </is>
       </c>
-      <c r="D17" s="28" t="inlineStr">
+      <c r="D19" s="66" t="inlineStr">
         <is>
           <t>Author Substack</t>
         </is>
       </c>
-      <c r="E17" s="29" t="inlineStr">
-        <is>
-          <t>English professor, author. Literary and theological intersection. Hidden gem potential when she's writing essays.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="40" customHeight="1">
-      <c r="A18" s="30" t="inlineStr">
+      <c r="E19" s="40" t="inlineStr">
+        <is>
+          <t>English professor. Literary and theological intersection. Hidden gem potential.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="36" customHeight="1">
+      <c r="A20" s="64" t="inlineStr">
         <is>
           <t>Tish Harrison Warren</t>
         </is>
       </c>
-      <c r="B18" s="18" t="inlineStr">
+      <c r="B20" s="65" t="inlineStr">
         <is>
           <t>Tier 3</t>
         </is>
       </c>
-      <c r="C18" s="18" t="inlineStr">
+      <c r="C20" s="65" t="inlineStr">
         <is>
           <t>1.00×</t>
         </is>
       </c>
-      <c r="D18" s="31" t="inlineStr">
+      <c r="D20" s="66" t="inlineStr">
         <is>
           <t>Author Substack</t>
         </is>
       </c>
-      <c r="E18" s="32" t="inlineStr">
-        <is>
-          <t>Anglican priest, NYT contributor. Thoughtful, liturgical, accessible. High hidden gem potential.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="40" customHeight="1">
-      <c r="A19" s="26" t="inlineStr">
+      <c r="E20" s="40" t="inlineStr">
+        <is>
+          <t>Anglican priest, NYT contributor. Thoughtful and liturgical. Hidden gem potential.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="36" customHeight="1">
+      <c r="A21" s="64" t="inlineStr">
         <is>
           <t>Jake Meador (Mere Orthodoxy)</t>
         </is>
       </c>
-      <c r="B19" s="18" t="inlineStr">
+      <c r="B21" s="65" t="inlineStr">
         <is>
           <t>Tier 3</t>
         </is>
       </c>
-      <c r="C19" s="18" t="inlineStr">
+      <c r="C21" s="65" t="inlineStr">
         <is>
           <t>1.00×</t>
         </is>
       </c>
-      <c r="D19" s="28" t="inlineStr">
+      <c r="D21" s="66" t="inlineStr">
         <is>
           <t>Author Substack</t>
         </is>
       </c>
-      <c r="E19" s="29" t="inlineStr">
-        <is>
-          <t>Editor of Mere Orthodoxy. Cultural and political theology. Excellent writer — apply hidden gem bonus liberally.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="40" customHeight="1">
-      <c r="A20" s="30" t="inlineStr">
+      <c r="E21" s="40" t="inlineStr">
+        <is>
+          <t>Editor of Mere Orthodoxy. Excellent writer — apply hidden gem bonus liberally.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="36" customHeight="1">
+      <c r="A22" s="64" t="inlineStr">
         <is>
           <t>Samuel James</t>
         </is>
       </c>
-      <c r="B20" s="18" t="inlineStr">
+      <c r="B22" s="65" t="inlineStr">
         <is>
           <t>Tier 3</t>
         </is>
       </c>
-      <c r="C20" s="18" t="inlineStr">
+      <c r="C22" s="65" t="inlineStr">
         <is>
           <t>1.00×</t>
         </is>
       </c>
-      <c r="D20" s="31" t="inlineStr">
+      <c r="D22" s="66" t="inlineStr">
         <is>
           <t>Author Substack</t>
         </is>
       </c>
-      <c r="E20" s="32" t="inlineStr">
-        <is>
-          <t>Christianity Today staff. Culture, technology, church. Very readable. High hidden gem potential.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="40" customHeight="1">
-      <c r="A21" s="26" t="inlineStr">
+      <c r="E22" s="40" t="inlineStr">
+        <is>
+          <t>Christianity Today staff. Culture, technology, church. High hidden gem potential.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="36" customHeight="1">
+      <c r="A23" s="64" t="inlineStr">
         <is>
           <t>Alan Jacobs</t>
         </is>
       </c>
-      <c r="B21" s="18" t="inlineStr">
+      <c r="B23" s="65" t="inlineStr">
         <is>
           <t>Tier 3</t>
         </is>
       </c>
-      <c r="C21" s="18" t="inlineStr">
+      <c r="C23" s="65" t="inlineStr">
         <is>
           <t>1.00×</t>
         </is>
       </c>
-      <c r="D21" s="28" t="inlineStr">
+      <c r="D23" s="66" t="inlineStr">
         <is>
           <t>Author Substack</t>
         </is>
       </c>
-      <c r="E21" s="29" t="inlineStr">
-        <is>
-          <t>Baylor professor, prolific essayist. Literary and theological. Consistently Tier 1 quality — hidden gem always applies.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="40" customHeight="1">
-      <c r="A22" s="30" t="inlineStr">
-        <is>
-          <t>Kyle Worley</t>
-        </is>
-      </c>
-      <c r="B22" s="18" t="inlineStr">
+      <c r="E23" s="40" t="inlineStr">
+        <is>
+          <t>Baylor professor. Literary and theological. Consistently Tier 1 quality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="36" customHeight="1">
+      <c r="A24" s="64" t="inlineStr">
+        <is>
+          <t>Carey Nieuwhof</t>
+        </is>
+      </c>
+      <c r="B24" s="65" t="inlineStr">
         <is>
           <t>Tier 3</t>
         </is>
       </c>
-      <c r="C22" s="18" t="inlineStr">
+      <c r="C24" s="65" t="inlineStr">
         <is>
           <t>1.00×</t>
         </is>
       </c>
-      <c r="D22" s="31" t="inlineStr">
+      <c r="D24" s="66" t="inlineStr">
         <is>
           <t>Author Substack</t>
         </is>
       </c>
-      <c r="E22" s="32" t="inlineStr">
-        <is>
-          <t>Pastor/theologian. Theologically solid, pastoral tone. Apply hidden gem when substantive.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="40" customHeight="1">
-      <c r="A23" s="26" t="inlineStr">
-        <is>
-          <t>Jen Wilkin</t>
-        </is>
-      </c>
-      <c r="B23" s="18" t="inlineStr">
-        <is>
-          <t>Tier 3</t>
-        </is>
-      </c>
-      <c r="C23" s="18" t="inlineStr">
-        <is>
-          <t>1.00×</t>
-        </is>
-      </c>
-      <c r="D23" s="28" t="inlineStr">
-        <is>
-          <t>Author Substack</t>
-        </is>
-      </c>
-      <c r="E23" s="29" t="inlineStr">
-        <is>
-          <t>Bible teacher, author. Strong on women's ministry and biblical literacy. Good for women and parent personas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="40" customHeight="1">
-      <c r="A24" s="30" t="inlineStr">
-        <is>
-          <t>Carey Nieuwhof</t>
-        </is>
-      </c>
-      <c r="B24" s="18" t="inlineStr">
-        <is>
-          <t>Tier 3</t>
-        </is>
-      </c>
-      <c r="C24" s="18" t="inlineStr">
-        <is>
-          <t>1.00×</t>
-        </is>
-      </c>
-      <c r="D24" s="31" t="inlineStr">
-        <is>
-          <t>Author Substack</t>
-        </is>
-      </c>
-      <c r="E24" s="32" t="inlineStr">
-        <is>
-          <t>Church leadership and ministry growth. Practical, pastoral. Best for pastor persona. Watch for promotional content.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="40" customHeight="1">
-      <c r="A25" s="26" t="inlineStr">
+      <c r="E24" s="40" t="inlineStr">
+        <is>
+          <t>Church leadership. Practical, pastoral. Watch for promotional content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="36" customHeight="1">
+      <c r="A25" s="67" t="inlineStr">
         <is>
           <t>BBC Religion</t>
         </is>
       </c>
-      <c r="B25" s="24" t="inlineStr">
+      <c r="B25" s="68" t="inlineStr">
         <is>
           <t>Tier 4</t>
         </is>
       </c>
-      <c r="C25" s="24" t="inlineStr">
+      <c r="C25" s="68" t="inlineStr">
         <is>
           <t>0.85×</t>
         </is>
       </c>
-      <c r="D25" s="28" t="inlineStr">
+      <c r="D25" s="69" t="inlineStr">
         <is>
           <t>World News</t>
         </is>
       </c>
-      <c r="E25" s="29" t="inlineStr">
-        <is>
-          <t>Solid religion reporting. Pre-filtered for Christian relevance. Use for major news stories touching Christianity.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="40" customHeight="1">
-      <c r="A26" s="30" t="inlineStr">
+      <c r="E25" s="70" t="inlineStr">
+        <is>
+          <t>Solid religion reporting. Use for major news stories touching Christianity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="36" customHeight="1">
+      <c r="A26" s="67" t="inlineStr">
         <is>
           <t>The New York Times</t>
         </is>
       </c>
-      <c r="B26" s="24" t="inlineStr">
+      <c r="B26" s="68" t="inlineStr">
         <is>
           <t>Tier 4</t>
         </is>
       </c>
-      <c r="C26" s="24" t="inlineStr">
+      <c r="C26" s="68" t="inlineStr">
         <is>
           <t>0.85×</t>
         </is>
       </c>
-      <c r="D26" s="31" t="inlineStr">
+      <c r="D26" s="69" t="inlineStr">
         <is>
           <t>World News</t>
         </is>
       </c>
-      <c r="E26" s="32" t="inlineStr">
-        <is>
-          <t>High-quality journalism but secular lens. Religion coverage is inconsistent. Filter carefully.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="40" customHeight="1">
-      <c r="A27" s="26" t="inlineStr">
+      <c r="E26" s="70" t="inlineStr">
+        <is>
+          <t>High-quality journalism but secular lens. Religion coverage inconsistent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="36" customHeight="1">
+      <c r="A27" s="67" t="inlineStr">
         <is>
           <t>The Guardian</t>
         </is>
       </c>
-      <c r="B27" s="24" t="inlineStr">
+      <c r="B27" s="68" t="inlineStr">
         <is>
           <t>Tier 4</t>
         </is>
       </c>
-      <c r="C27" s="24" t="inlineStr">
+      <c r="C27" s="68" t="inlineStr">
         <is>
           <t>0.85×</t>
         </is>
       </c>
-      <c r="D27" s="28" t="inlineStr">
+      <c r="D27" s="69" t="inlineStr">
         <is>
           <t>World News</t>
         </is>
       </c>
-      <c r="E27" s="29" t="inlineStr">
-        <is>
-          <t>Left-leaning. Religion coverage often critical of Christianity. Useful for understanding cultural moment.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="40" customHeight="1">
-      <c r="A28" s="30" t="inlineStr">
+      <c r="E27" s="70" t="inlineStr">
+        <is>
+          <t>Left-leaning. Religion coverage often critical. Useful for cultural context.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="36" customHeight="1">
+      <c r="A28" s="67" t="inlineStr">
         <is>
           <t>Associated Press</t>
         </is>
       </c>
-      <c r="B28" s="24" t="inlineStr">
+      <c r="B28" s="68" t="inlineStr">
         <is>
           <t>Tier 4</t>
         </is>
       </c>
-      <c r="C28" s="24" t="inlineStr">
+      <c r="C28" s="68" t="inlineStr">
         <is>
           <t>0.85×</t>
         </is>
       </c>
-      <c r="D28" s="31" t="inlineStr">
+      <c r="D28" s="69" t="inlineStr">
         <is>
           <t>World News</t>
         </is>
       </c>
-      <c r="E28" s="32" t="inlineStr">
-        <is>
-          <t>Wire service. Factual, neutral. Good for breaking news with Christian angle (persecution, legislation, etc.).</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="40" customHeight="1">
-      <c r="A29" s="26" t="inlineStr">
+      <c r="E28" s="70" t="inlineStr">
+        <is>
+          <t>Wire service. Factual, neutral. Good for breaking news with Christian angle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="36" customHeight="1">
+      <c r="A29" s="67" t="inlineStr">
         <is>
           <t>Washington Post</t>
         </is>
       </c>
-      <c r="B29" s="24" t="inlineStr">
+      <c r="B29" s="68" t="inlineStr">
         <is>
           <t>Tier 4</t>
         </is>
       </c>
-      <c r="C29" s="24" t="inlineStr">
+      <c r="C29" s="68" t="inlineStr">
         <is>
           <t>0.85×</t>
         </is>
       </c>
-      <c r="D29" s="28" t="inlineStr">
+      <c r="D29" s="69" t="inlineStr">
         <is>
           <t>World News</t>
         </is>
       </c>
-      <c r="E29" s="29" t="inlineStr">
-        <is>
-          <t>Quality journalism, secular perspective. Religion section worth monitoring for major stories.</t>
+      <c r="E29" s="70" t="inlineStr">
+        <is>
+          <t>Quality journalism, secular perspective. Monitor for major religion stories.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add recency penalty for old articles; update source tiers and world news feeds
- Hard cutoff: drop articles older than 30 days entirely
- Recency penalties: -2.0 (3-7d), -4.0 (7-14d), -6.0 (14-30d)
- Fixes 2021 Jen Wilkin article and 2011 9Marks article surfacing in digest
- Add WSJ, AP Top News, BBC World, NYT World as sources
- Per-tier source caps: Tier 1/1A=5, Tier 2=3, Tier 3/4=2
- World news tiers: AP/BBC/NYT/WSJ=0.90x, Guardian/WaPo=0.80x
- Add Top World Story flagging in email and site
- Update scoring_algorithm.xlsx with Rule 9 (Recency Penalties)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scoring_algorithm.xlsx
+++ b/scoring_algorithm.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -86,8 +86,34 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00CC0000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00555555"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -157,6 +183,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="008B4513"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E8DA"/>
       </patternFill>
     </fill>
   </fills>
@@ -230,7 +261,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -436,6 +467,27 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -803,7 +855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D65"/>
+  <dimension ref="A1:D75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1639,6 +1691,122 @@
         </is>
       </c>
       <c r="D65" s="7" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="71" t="inlineStr">
+        <is>
+          <t>9. RECENCY PENALTIES (OLD ARTICLES)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="72" t="inlineStr">
+        <is>
+          <t>Age of Article</t>
+        </is>
+      </c>
+      <c r="B68" s="72" t="inlineStr">
+        <is>
+          <t>Penalty</t>
+        </is>
+      </c>
+      <c r="C68" s="72" t="inlineStr">
+        <is>
+          <t>Definition</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="73" t="inlineStr">
+        <is>
+          <t>0–72 hours</t>
+        </is>
+      </c>
+      <c r="B69" s="74" t="inlineStr">
+        <is>
+          <t>+0.25 to +1.5</t>
+        </is>
+      </c>
+      <c r="C69" s="75" t="inlineStr">
+        <is>
+          <t>Recency BOOST (see Rule 3). Articles within 72h are rewarded for freshness.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="73" t="inlineStr">
+        <is>
+          <t>3–7 days</t>
+        </is>
+      </c>
+      <c r="B70" s="74" t="inlineStr">
+        <is>
+          <t>−2.0</t>
+        </is>
+      </c>
+      <c r="C70" s="75" t="inlineStr">
+        <is>
+          <t>Article is showing its age. Still potentially useful but deprioritised. Will rarely surface unless content score is very high.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="73" t="inlineStr">
+        <is>
+          <t>7–14 days</t>
+        </is>
+      </c>
+      <c r="B71" s="74" t="inlineStr">
+        <is>
+          <t>−4.0</t>
+        </is>
+      </c>
+      <c r="C71" s="75" t="inlineStr">
+        <is>
+          <t>Significant staleness penalty. Article would need a 9+ AI score to break into the top 10 after this penalty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="73" t="inlineStr">
+        <is>
+          <t>14–30 days</t>
+        </is>
+      </c>
+      <c r="B72" s="74" t="inlineStr">
+        <is>
+          <t>−6.0</t>
+        </is>
+      </c>
+      <c r="C72" s="75" t="inlineStr">
+        <is>
+          <t>Near-suppression. Only extraordinary content (score 10) would survive. Effectively excluded from the digest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="73" t="inlineStr">
+        <is>
+          <t>30+ days</t>
+        </is>
+      </c>
+      <c r="B73" s="76" t="inlineStr">
+        <is>
+          <t>HARD DROP</t>
+        </is>
+      </c>
+      <c r="C73" s="75" t="inlineStr">
+        <is>
+          <t>Hard cutoff. Articles older than 30 days are excluded entirely from the pipeline before scoring. This prevents evergreen/undated RSS content from recycling indefinitely.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="77" t="inlineStr">
+        <is>
+          <t>Note: The hard 30-day cutoff was added after a 2021 Jen Wilkin article and a 2011 9Marks article appeared in the digest. RSS feeds sometimes surface evergreen posts; this cutoff prevents them from recycling.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="54">
@@ -1707,7 +1875,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1731,6 +1899,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2306,12 +2475,12 @@
       </c>
       <c r="B25" s="68" t="inlineStr">
         <is>
-          <t>Tier 4</t>
+          <t>Tier 4A</t>
         </is>
       </c>
       <c r="C25" s="68" t="inlineStr">
         <is>
-          <t>0.85×</t>
+          <t>0.90×</t>
         </is>
       </c>
       <c r="D25" s="69" t="inlineStr">
@@ -2333,12 +2502,12 @@
       </c>
       <c r="B26" s="68" t="inlineStr">
         <is>
-          <t>Tier 4</t>
+          <t>Tier 4A</t>
         </is>
       </c>
       <c r="C26" s="68" t="inlineStr">
         <is>
-          <t>0.85×</t>
+          <t>0.90×</t>
         </is>
       </c>
       <c r="D26" s="69" t="inlineStr">
@@ -2360,12 +2529,12 @@
       </c>
       <c r="B27" s="68" t="inlineStr">
         <is>
-          <t>Tier 4</t>
+          <t>Tier 4B</t>
         </is>
       </c>
       <c r="C27" s="68" t="inlineStr">
         <is>
-          <t>0.85×</t>
+          <t>0.80×</t>
         </is>
       </c>
       <c r="D27" s="69" t="inlineStr">
@@ -2387,12 +2556,12 @@
       </c>
       <c r="B28" s="68" t="inlineStr">
         <is>
-          <t>Tier 4</t>
+          <t>Tier 4A</t>
         </is>
       </c>
       <c r="C28" s="68" t="inlineStr">
         <is>
-          <t>0.85×</t>
+          <t>0.90×</t>
         </is>
       </c>
       <c r="D28" s="69" t="inlineStr">
@@ -2414,12 +2583,12 @@
       </c>
       <c r="B29" s="68" t="inlineStr">
         <is>
-          <t>Tier 4</t>
+          <t>Tier 4B</t>
         </is>
       </c>
       <c r="C29" s="68" t="inlineStr">
         <is>
-          <t>0.85×</t>
+          <t>0.80×</t>
         </is>
       </c>
       <c r="D29" s="69" t="inlineStr">
@@ -2430,6 +2599,114 @@
       <c r="E29" s="70" t="inlineStr">
         <is>
           <t>Quality journalism, secular perspective. Monitor for major religion stories.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="75" t="inlineStr">
+        <is>
+          <t>Associated Press Religion</t>
+        </is>
+      </c>
+      <c r="B30" s="75" t="inlineStr">
+        <is>
+          <t>Tier 4A</t>
+        </is>
+      </c>
+      <c r="C30" s="75" t="inlineStr">
+        <is>
+          <t>0.90×</t>
+        </is>
+      </c>
+      <c r="D30" s="75" t="inlineStr">
+        <is>
+          <t>World News</t>
+        </is>
+      </c>
+      <c r="E30" s="75" t="inlineStr">
+        <is>
+          <t>AP Religion feed — same wire quality as AP Top News. Focused on religion stories with a Christian angle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="75" t="inlineStr">
+        <is>
+          <t>BBC News</t>
+        </is>
+      </c>
+      <c r="B31" s="75" t="inlineStr">
+        <is>
+          <t>Tier 4A</t>
+        </is>
+      </c>
+      <c r="C31" s="75" t="inlineStr">
+        <is>
+          <t>0.90×</t>
+        </is>
+      </c>
+      <c r="D31" s="75" t="inlineStr">
+        <is>
+          <t>World News</t>
+        </is>
+      </c>
+      <c r="E31" s="75" t="inlineStr">
+        <is>
+          <t>BBC World News feed. High-quality international journalism. 0.90x tier for factual, non-perspective-driven reporting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="75" t="inlineStr">
+        <is>
+          <t>The New York Times Religion</t>
+        </is>
+      </c>
+      <c r="B32" s="75" t="inlineStr">
+        <is>
+          <t>Tier 4A</t>
+        </is>
+      </c>
+      <c r="C32" s="75" t="inlineStr">
+        <is>
+          <t>0.90×</t>
+        </is>
+      </c>
+      <c r="D32" s="75" t="inlineStr">
+        <is>
+          <t>World News</t>
+        </is>
+      </c>
+      <c r="E32" s="75" t="inlineStr">
+        <is>
+          <t>NYT Religion section — more focused than the general World feed. Useful for major religion stories.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="75" t="inlineStr">
+        <is>
+          <t>Wall Street Journal</t>
+        </is>
+      </c>
+      <c r="B33" s="75" t="inlineStr">
+        <is>
+          <t>Tier 4A</t>
+        </is>
+      </c>
+      <c r="C33" s="75" t="inlineStr">
+        <is>
+          <t>0.90×</t>
+        </is>
+      </c>
+      <c r="D33" s="75" t="inlineStr">
+        <is>
+          <t>World News</t>
+        </is>
+      </c>
+      <c r="E33" s="75" t="inlineStr">
+        <is>
+          <t>WSJ World News. Elevated above Guardian/WaPo for fact-first reporting quality. Less religion-specific but strong for major world events.</t>
         </is>
       </c>
     </row>

</xml_diff>